<commit_message>
feat: Add Dockerfile and requirements, and update prediction charts, Excel output, and model report with refined metrics.
</commit_message>
<xml_diff>
--- a/output/predictions_2026.xlsx
+++ b/output/predictions_2026.xlsx
@@ -749,7 +749,7 @@
         <v>185276829.8694343</v>
       </c>
       <c r="C3" s="6">
-        <v>623553080.8921326</v>
+        <v>623553080.8921325</v>
       </c>
       <c r="D3" s="6">
         <v>126038610</v>
@@ -795,7 +795,7 @@
         <v>191354420.5233864</v>
       </c>
       <c r="C5" s="6">
-        <v>593356855.0657954</v>
+        <v>593356855.0657955</v>
       </c>
       <c r="D5" s="6">
         <v>42004996</v>
@@ -838,7 +838,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="6">
-        <v>198592010.9299968</v>
+        <v>198592010.9299969</v>
       </c>
       <c r="C7" s="6">
         <v>595807228.4087459</v>
@@ -864,7 +864,7 @@
         <v>201950379.0522418</v>
       </c>
       <c r="C8" s="3">
-        <v>635727944.3552259</v>
+        <v>635727944.355226</v>
       </c>
       <c r="D8" s="3">
         <v>51324340</v>
@@ -887,7 +887,7 @@
         <v>203881927.8084632</v>
       </c>
       <c r="C9" s="6">
-        <v>614936723.3479046</v>
+        <v>614936723.3479044</v>
       </c>
       <c r="D9" s="6">
         <v>271446755</v>
@@ -907,10 +907,10 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>213738222.1960625</v>
+        <v>213738222.1960626</v>
       </c>
       <c r="C10" s="3">
-        <v>629765991.3898178</v>
+        <v>629765991.389818</v>
       </c>
       <c r="D10" s="3">
         <v>116429626</v>
@@ -933,7 +933,7 @@
         <v>220174987.2432342</v>
       </c>
       <c r="C11" s="6">
-        <v>620204708.7153965</v>
+        <v>620204708.7153964</v>
       </c>
       <c r="D11" s="6">
         <v>193586314</v>
@@ -956,7 +956,7 @@
         <v>241573210.0778116</v>
       </c>
       <c r="C12" s="3">
-        <v>592308158.0984476</v>
+        <v>592308158.0984477</v>
       </c>
       <c r="D12" s="3">
         <v>135212500</v>
@@ -976,7 +976,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="6">
-        <v>259941164.6040252</v>
+        <v>259941164.6040253</v>
       </c>
       <c r="C13" s="6">
         <v>608075627.3723929</v>
@@ -1002,7 +1002,7 @@
         <v>2475771754.766472</v>
       </c>
       <c r="C14" s="9">
-        <v>7303917893.15903</v>
+        <v>7303917893.159029</v>
       </c>
       <c r="D14" s="9">
         <v>1962149005</v>
@@ -1014,7 +1014,7 @@
         <v>0.2617654156017943</v>
       </c>
       <c r="G14" s="10">
-        <v>0.1192424021739156</v>
+        <v>0.1192424021739154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>